<commit_message>
Added ventilator validation patient
</commit_message>
<xml_diff>
--- a/data/Data.xlsx
+++ b/data/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC6A2E9E-4B1F-4A80-872F-6A32EDC10C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{687CD05D-E31A-4B86-B6F4-991420C95501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27315" yWindow="4230" windowWidth="23685" windowHeight="24570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="26460" yWindow="2205" windowWidth="26100" windowHeight="24405" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patients" sheetId="6" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5501" uniqueCount="799">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5491" uniqueCount="805">
   <si>
     <t>Name</t>
   </si>
@@ -2447,6 +2447,24 @@
   </si>
   <si>
     <t>74 in</t>
+  </si>
+  <si>
+    <t>Ventilated</t>
+  </si>
+  <si>
+    <t>64.35 in</t>
+  </si>
+  <si>
+    <t>Aorta</t>
+  </si>
+  <si>
+    <t>PartialPressure</t>
+  </si>
+  <si>
+    <t>7200 s</t>
+  </si>
+  <si>
+    <t>300 s</t>
   </si>
 </sst>
 </file>
@@ -3829,7 +3847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB26"/>
+  <dimension ref="A1:AC26"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.5703125" style="117" bestFit="1" customWidth="1"/>
@@ -3839,22 +3857,22 @@
     <col min="5" max="5" width="14.28515625" style="121" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.42578125" style="121" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.28515625" style="121" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" style="121" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" style="121" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" style="121" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="121" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.140625" style="121" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" style="121" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.140625" style="121" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" style="121" bestFit="1" customWidth="1"/>
-    <col min="16" max="19" width="10.7109375" style="121" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.140625" style="121" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.85546875" style="121" bestFit="1" customWidth="1"/>
-    <col min="22" max="28" width="15.85546875" style="121" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="8.85546875" style="121"/>
+    <col min="8" max="9" width="12.42578125" style="121" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" style="121" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" style="121" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="121" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.140625" style="121" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" style="121" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.140625" style="121" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" style="121" bestFit="1" customWidth="1"/>
+    <col min="17" max="20" width="10.7109375" style="121" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.140625" style="121" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.85546875" style="121" bestFit="1" customWidth="1"/>
+    <col min="23" max="29" width="15.85546875" style="121" bestFit="1" customWidth="1"/>
+    <col min="30" max="16384" width="8.85546875" style="121"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="116"/>
       <c r="B1" s="156" t="s">
         <v>583</v>
@@ -3867,11 +3885,11 @@
       </c>
       <c r="G1" s="157"/>
       <c r="H1" s="157"/>
-      <c r="I1" s="158"/>
-      <c r="J1" s="156" t="s">
+      <c r="I1" s="157"/>
+      <c r="J1" s="158"/>
+      <c r="K1" s="156" t="s">
         <v>581</v>
       </c>
-      <c r="K1" s="157"/>
       <c r="L1" s="157"/>
       <c r="M1" s="157"/>
       <c r="N1" s="157"/>
@@ -3879,22 +3897,23 @@
       <c r="P1" s="157"/>
       <c r="Q1" s="157"/>
       <c r="R1" s="157"/>
-      <c r="S1" s="158"/>
-      <c r="T1" s="156" t="s">
+      <c r="S1" s="157"/>
+      <c r="T1" s="158"/>
+      <c r="U1" s="156" t="s">
         <v>582</v>
       </c>
-      <c r="U1" s="158"/>
-      <c r="V1" s="156" t="s">
+      <c r="V1" s="158"/>
+      <c r="W1" s="156" t="s">
         <v>780</v>
       </c>
-      <c r="W1" s="157"/>
       <c r="X1" s="157"/>
       <c r="Y1" s="157"/>
       <c r="Z1" s="157"/>
       <c r="AA1" s="157"/>
-      <c r="AB1" s="158"/>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB1" s="157"/>
+      <c r="AC1" s="158"/>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" s="117" t="s">
         <v>0</v>
       </c>
@@ -3919,68 +3938,71 @@
       <c r="H2" s="118" t="s">
         <v>609</v>
       </c>
-      <c r="I2" s="126" t="s">
+      <c r="I2" s="118" t="s">
         <v>610</v>
       </c>
-      <c r="J2" s="125" t="s">
+      <c r="J2" s="126" t="s">
+        <v>799</v>
+      </c>
+      <c r="K2" s="125" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="118" t="s">
+      <c r="L2" s="118" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="118" t="s">
+      <c r="M2" s="118" t="s">
         <v>27</v>
       </c>
-      <c r="M2" s="118" t="s">
+      <c r="N2" s="118" t="s">
         <v>28</v>
       </c>
-      <c r="N2" s="118" t="s">
+      <c r="O2" s="118" t="s">
         <v>29</v>
       </c>
-      <c r="O2" s="118" t="s">
+      <c r="P2" s="118" t="s">
         <v>70</v>
       </c>
-      <c r="P2" s="118" t="s">
+      <c r="Q2" s="118" t="s">
         <v>68</v>
       </c>
-      <c r="Q2" s="118" t="s">
+      <c r="R2" s="118" t="s">
         <v>300</v>
       </c>
-      <c r="R2" s="118" t="s">
+      <c r="S2" s="118" t="s">
         <v>303</v>
       </c>
-      <c r="S2" s="126" t="s">
+      <c r="T2" s="126" t="s">
         <v>307</v>
       </c>
-      <c r="T2" s="125" t="s">
+      <c r="U2" s="125" t="s">
         <v>574</v>
       </c>
-      <c r="U2" s="126" t="s">
+      <c r="V2" s="126" t="s">
         <v>575</v>
       </c>
-      <c r="V2" s="125" t="s">
+      <c r="W2" s="125" t="s">
         <v>781</v>
       </c>
-      <c r="W2" s="125" t="s">
+      <c r="X2" s="125" t="s">
         <v>782</v>
       </c>
-      <c r="X2" s="125" t="s">
+      <c r="Y2" s="125" t="s">
         <v>783</v>
       </c>
-      <c r="Y2" s="125" t="s">
+      <c r="Z2" s="125" t="s">
         <v>784</v>
       </c>
-      <c r="Z2" s="125" t="s">
+      <c r="AA2" s="125" t="s">
         <v>785</v>
       </c>
-      <c r="AA2" s="125" t="s">
+      <c r="AB2" s="125" t="s">
         <v>786</v>
       </c>
-      <c r="AB2" s="125" t="s">
+      <c r="AC2" s="125" t="s">
         <v>787</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="116" t="s">
         <v>562</v>
       </c>
@@ -3991,9 +4013,9 @@
       <c r="F3" s="127"/>
       <c r="G3" s="122"/>
       <c r="H3" s="122"/>
-      <c r="I3" s="128"/>
-      <c r="J3" s="127"/>
-      <c r="K3" s="122"/>
+      <c r="I3" s="122"/>
+      <c r="J3" s="128"/>
+      <c r="K3" s="127"/>
       <c r="L3" s="122"/>
       <c r="M3" s="122"/>
       <c r="N3" s="122"/>
@@ -4001,18 +4023,19 @@
       <c r="P3" s="122"/>
       <c r="Q3" s="122"/>
       <c r="R3" s="122"/>
-      <c r="S3" s="128"/>
-      <c r="T3" s="127"/>
-      <c r="U3" s="128"/>
-      <c r="V3" s="127"/>
-      <c r="W3" s="122"/>
+      <c r="S3" s="122"/>
+      <c r="T3" s="128"/>
+      <c r="U3" s="127"/>
+      <c r="V3" s="128"/>
+      <c r="W3" s="127"/>
       <c r="X3" s="122"/>
       <c r="Y3" s="122"/>
       <c r="Z3" s="122"/>
       <c r="AA3" s="122"/>
-      <c r="AB3" s="128"/>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB3" s="122"/>
+      <c r="AC3" s="128"/>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="123" t="s">
         <v>409</v>
       </c>
@@ -4037,14 +4060,14 @@
       <c r="H4" s="119" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="119" t="s">
         <v>9</v>
       </c>
-      <c r="J4" s="129" t="s">
+      <c r="J4" s="130" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4" s="129" t="s">
         <v>30</v>
-      </c>
-      <c r="K4" s="119" t="s">
-        <v>9</v>
       </c>
       <c r="L4" s="119" t="s">
         <v>9</v>
@@ -4065,40 +4088,43 @@
         <v>9</v>
       </c>
       <c r="R4" s="119" t="s">
+        <v>9</v>
+      </c>
+      <c r="S4" s="119" t="s">
         <v>30</v>
       </c>
-      <c r="S4" s="130" t="s">
+      <c r="T4" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="T4" s="129" t="s">
+      <c r="U4" s="129" t="s">
         <v>30</v>
       </c>
-      <c r="U4" s="130" t="s">
-        <v>9</v>
-      </c>
-      <c r="V4" s="129" t="s">
+      <c r="V4" s="130" t="s">
         <v>9</v>
       </c>
       <c r="W4" s="129" t="s">
         <v>9</v>
       </c>
       <c r="X4" s="129" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y4" s="129" t="s">
         <v>30</v>
       </c>
-      <c r="Y4" s="129" t="s">
+      <c r="Z4" s="129" t="s">
         <v>9</v>
       </c>
-      <c r="Z4" s="129" t="s">
+      <c r="AA4" s="129" t="s">
         <v>30</v>
-      </c>
-      <c r="AA4" s="129" t="s">
-        <v>9</v>
       </c>
       <c r="AB4" s="129" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC4" s="129" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="116" t="s">
         <v>590</v>
       </c>
@@ -4109,9 +4135,9 @@
       <c r="F5" s="127"/>
       <c r="G5" s="122"/>
       <c r="H5" s="122"/>
-      <c r="I5" s="128"/>
-      <c r="J5" s="127"/>
-      <c r="K5" s="122"/>
+      <c r="I5" s="122"/>
+      <c r="J5" s="128"/>
+      <c r="K5" s="127"/>
       <c r="L5" s="122"/>
       <c r="M5" s="122"/>
       <c r="N5" s="122"/>
@@ -4119,18 +4145,19 @@
       <c r="P5" s="122"/>
       <c r="Q5" s="122"/>
       <c r="R5" s="122"/>
-      <c r="S5" s="128"/>
-      <c r="T5" s="127"/>
-      <c r="U5" s="128"/>
-      <c r="V5" s="127"/>
-      <c r="W5" s="122"/>
+      <c r="S5" s="122"/>
+      <c r="T5" s="128"/>
+      <c r="U5" s="127"/>
+      <c r="V5" s="128"/>
+      <c r="W5" s="127"/>
       <c r="X5" s="122"/>
       <c r="Y5" s="122"/>
       <c r="Z5" s="122"/>
       <c r="AA5" s="122"/>
-      <c r="AB5" s="128"/>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB5" s="122"/>
+      <c r="AC5" s="128"/>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="124" t="s">
         <v>5</v>
       </c>
@@ -4151,68 +4178,71 @@
       <c r="H6" s="120" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="132" t="s">
+      <c r="I6" s="120" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="131" t="s">
+      <c r="J6" s="132" t="s">
+        <v>795</v>
+      </c>
+      <c r="K6" s="131" t="s">
         <v>31</v>
       </c>
-      <c r="K6" s="120" t="s">
+      <c r="L6" s="120" t="s">
         <v>32</v>
-      </c>
-      <c r="L6" s="120" t="s">
-        <v>19</v>
       </c>
       <c r="M6" s="120" t="s">
         <v>19</v>
       </c>
       <c r="N6" s="120" t="s">
+        <v>19</v>
+      </c>
+      <c r="O6" s="120" t="s">
         <v>33</v>
       </c>
-      <c r="O6" s="120" t="s">
+      <c r="P6" s="120" t="s">
         <v>34</v>
       </c>
-      <c r="P6" s="120" t="s">
+      <c r="Q6" s="120" t="s">
         <v>299</v>
       </c>
-      <c r="Q6" s="120" t="s">
+      <c r="R6" s="120" t="s">
         <v>301</v>
       </c>
-      <c r="R6" s="120" t="s">
+      <c r="S6" s="120" t="s">
         <v>304</v>
       </c>
-      <c r="S6" s="132" t="s">
+      <c r="T6" s="132" t="s">
         <v>566</v>
       </c>
-      <c r="T6" s="131" t="s">
+      <c r="U6" s="131" t="s">
         <v>566</v>
       </c>
-      <c r="U6" s="132" t="s">
+      <c r="V6" s="132" t="s">
         <v>577</v>
       </c>
-      <c r="V6" s="131" t="s">
+      <c r="W6" s="131" t="s">
         <v>299</v>
       </c>
-      <c r="W6" s="120" t="s">
+      <c r="X6" s="120" t="s">
         <v>795</v>
-      </c>
-      <c r="X6" s="120" t="s">
-        <v>301</v>
       </c>
       <c r="Y6" s="120" t="s">
         <v>301</v>
       </c>
       <c r="Z6" s="120" t="s">
+        <v>301</v>
+      </c>
+      <c r="AA6" s="120" t="s">
         <v>34</v>
       </c>
-      <c r="AA6" s="120" t="s">
+      <c r="AB6" s="120" t="s">
         <v>33</v>
       </c>
-      <c r="AB6" s="132" t="s">
+      <c r="AC6" s="132" t="s">
         <v>789</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="124" t="s">
         <v>6</v>
       </c>
@@ -4233,64 +4263,65 @@
       <c r="H7" s="120" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="132" t="s">
+      <c r="I7" s="120" t="s">
         <v>21</v>
       </c>
-      <c r="J7" s="131" t="s">
+      <c r="J7" s="132"/>
+      <c r="K7" s="131" t="s">
         <v>74</v>
       </c>
-      <c r="K7" s="120" t="s">
+      <c r="L7" s="120" t="s">
         <v>36</v>
-      </c>
-      <c r="L7" s="120" t="s">
-        <v>21</v>
       </c>
       <c r="M7" s="120" t="s">
         <v>21</v>
       </c>
       <c r="N7" s="120" t="s">
+        <v>21</v>
+      </c>
+      <c r="O7" s="120" t="s">
         <v>37</v>
       </c>
-      <c r="O7" s="120" t="s">
+      <c r="P7" s="120" t="s">
         <v>35</v>
       </c>
-      <c r="P7" s="120" t="s">
+      <c r="Q7" s="120" t="s">
         <v>21</v>
       </c>
-      <c r="Q7" s="120" t="s">
+      <c r="R7" s="120" t="s">
         <v>302</v>
       </c>
-      <c r="R7" s="120" t="s">
+      <c r="S7" s="120" t="s">
         <v>305</v>
       </c>
-      <c r="S7" s="132" t="s">
+      <c r="T7" s="132" t="s">
         <v>308</v>
       </c>
-      <c r="T7" s="131"/>
-      <c r="U7" s="132"/>
-      <c r="V7" s="131" t="s">
+      <c r="U7" s="131"/>
+      <c r="V7" s="132"/>
+      <c r="W7" s="131" t="s">
         <v>797</v>
       </c>
-      <c r="W7" s="120" t="s">
+      <c r="X7" s="120" t="s">
         <v>796</v>
-      </c>
-      <c r="X7" s="120" t="s">
-        <v>21</v>
       </c>
       <c r="Y7" s="120" t="s">
         <v>21</v>
       </c>
       <c r="Z7" s="120" t="s">
+        <v>21</v>
+      </c>
+      <c r="AA7" s="120" t="s">
         <v>791</v>
       </c>
-      <c r="AA7" s="120" t="s">
+      <c r="AB7" s="120" t="s">
         <v>573</v>
       </c>
-      <c r="AB7" s="132" t="s">
+      <c r="AC7" s="132" t="s">
         <v>788</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="124" t="s">
         <v>7</v>
       </c>
@@ -4311,68 +4342,71 @@
       <c r="H8" s="120" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="132" t="s">
+      <c r="I8" s="120" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="131" t="s">
+      <c r="J8" s="132" t="s">
+        <v>800</v>
+      </c>
+      <c r="K8" s="131" t="s">
         <v>39</v>
       </c>
-      <c r="K8" s="120" t="s">
+      <c r="L8" s="120" t="s">
         <v>42</v>
-      </c>
-      <c r="L8" s="120" t="s">
-        <v>20</v>
       </c>
       <c r="M8" s="120" t="s">
         <v>20</v>
       </c>
       <c r="N8" s="120" t="s">
+        <v>20</v>
+      </c>
+      <c r="O8" s="120" t="s">
         <v>40</v>
       </c>
-      <c r="O8" s="120" t="s">
+      <c r="P8" s="120" t="s">
         <v>38</v>
       </c>
-      <c r="P8" s="120" t="s">
+      <c r="Q8" s="120" t="s">
         <v>20</v>
       </c>
-      <c r="Q8" s="120" t="s">
+      <c r="R8" s="120" t="s">
         <v>38</v>
       </c>
-      <c r="R8" s="120" t="s">
+      <c r="S8" s="120" t="s">
         <v>306</v>
       </c>
-      <c r="S8" s="132" t="s">
+      <c r="T8" s="132" t="s">
         <v>39</v>
       </c>
-      <c r="T8" s="131" t="s">
+      <c r="U8" s="131" t="s">
         <v>578</v>
       </c>
-      <c r="U8" s="132" t="s">
+      <c r="V8" s="132" t="s">
         <v>579</v>
       </c>
-      <c r="V8" s="131" t="s">
+      <c r="W8" s="131" t="s">
         <v>798</v>
       </c>
-      <c r="W8" s="120" t="s">
+      <c r="X8" s="120" t="s">
         <v>793</v>
       </c>
-      <c r="X8" s="120" t="s">
+      <c r="Y8" s="120" t="s">
         <v>794</v>
       </c>
-      <c r="Y8" s="120" t="s">
+      <c r="Z8" s="120" t="s">
         <v>793</v>
       </c>
-      <c r="Z8" s="120" t="s">
+      <c r="AA8" s="120" t="s">
         <v>792</v>
       </c>
-      <c r="AA8" s="120" t="s">
+      <c r="AB8" s="120" t="s">
         <v>790</v>
       </c>
-      <c r="AB8" s="132" t="s">
+      <c r="AC8" s="132" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="124" t="s">
         <v>162</v>
       </c>
@@ -4393,13 +4427,11 @@
       <c r="H9" s="120">
         <v>0.18</v>
       </c>
-      <c r="I9" s="132">
+      <c r="I9" s="120">
         <v>0.18</v>
       </c>
-      <c r="J9" s="131">
-        <v>0.18</v>
-      </c>
-      <c r="K9" s="120">
+      <c r="J9" s="132"/>
+      <c r="K9" s="131">
         <v>0.18</v>
       </c>
       <c r="L9" s="120">
@@ -4418,29 +4450,32 @@
         <v>0.18</v>
       </c>
       <c r="Q9" s="120">
+        <v>0.18</v>
+      </c>
+      <c r="R9" s="120">
         <v>0.12</v>
       </c>
-      <c r="R9" s="120">
+      <c r="S9" s="120">
         <v>0.25</v>
       </c>
-      <c r="S9" s="132">
+      <c r="T9" s="132">
         <v>0.18</v>
       </c>
-      <c r="T9" s="131">
+      <c r="U9" s="131">
         <v>0.32</v>
       </c>
-      <c r="U9" s="132">
+      <c r="V9" s="132">
         <v>0.02</v>
       </c>
-      <c r="V9" s="131"/>
-      <c r="W9" s="120"/>
+      <c r="W9" s="131"/>
       <c r="X9" s="120"/>
       <c r="Y9" s="120"/>
       <c r="Z9" s="120"/>
       <c r="AA9" s="120"/>
-      <c r="AB9" s="132"/>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB9" s="120"/>
+      <c r="AC9" s="132"/>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="116" t="s">
         <v>591</v>
       </c>
@@ -4451,9 +4486,9 @@
       <c r="F10" s="127"/>
       <c r="G10" s="122"/>
       <c r="H10" s="122"/>
-      <c r="I10" s="128"/>
-      <c r="J10" s="127"/>
-      <c r="K10" s="122"/>
+      <c r="I10" s="122"/>
+      <c r="J10" s="128"/>
+      <c r="K10" s="127"/>
       <c r="L10" s="122"/>
       <c r="M10" s="122"/>
       <c r="N10" s="122"/>
@@ -4461,18 +4496,19 @@
       <c r="P10" s="122"/>
       <c r="Q10" s="122"/>
       <c r="R10" s="122"/>
-      <c r="S10" s="128"/>
-      <c r="T10" s="127"/>
-      <c r="U10" s="128"/>
-      <c r="V10" s="127"/>
-      <c r="W10" s="122"/>
+      <c r="S10" s="122"/>
+      <c r="T10" s="128"/>
+      <c r="U10" s="127"/>
+      <c r="V10" s="128"/>
+      <c r="W10" s="127"/>
       <c r="X10" s="122"/>
       <c r="Y10" s="122"/>
       <c r="Z10" s="122"/>
       <c r="AA10" s="122"/>
-      <c r="AB10" s="128"/>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB10" s="122"/>
+      <c r="AC10" s="128"/>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="124" t="s">
         <v>589</v>
       </c>
@@ -4483,9 +4519,9 @@
       <c r="F11" s="131"/>
       <c r="G11" s="120"/>
       <c r="H11" s="120"/>
-      <c r="I11" s="132"/>
-      <c r="J11" s="131"/>
-      <c r="K11" s="120"/>
+      <c r="I11" s="120"/>
+      <c r="J11" s="132"/>
+      <c r="K11" s="131"/>
       <c r="L11" s="120"/>
       <c r="M11" s="120"/>
       <c r="N11" s="120"/>
@@ -4493,18 +4529,19 @@
       <c r="P11" s="120"/>
       <c r="Q11" s="120"/>
       <c r="R11" s="120"/>
-      <c r="S11" s="132"/>
-      <c r="T11" s="131"/>
-      <c r="U11" s="132"/>
-      <c r="V11" s="131"/>
-      <c r="W11" s="120"/>
+      <c r="S11" s="120"/>
+      <c r="T11" s="132"/>
+      <c r="U11" s="131"/>
+      <c r="V11" s="132"/>
+      <c r="W11" s="131"/>
       <c r="X11" s="120"/>
       <c r="Y11" s="120"/>
       <c r="Z11" s="120"/>
       <c r="AA11" s="120"/>
-      <c r="AB11" s="132"/>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB11" s="120"/>
+      <c r="AC11" s="132"/>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="124" t="s">
         <v>555</v>
       </c>
@@ -4515,9 +4552,9 @@
       <c r="F12" s="131"/>
       <c r="G12" s="120"/>
       <c r="H12" s="120"/>
-      <c r="I12" s="132"/>
-      <c r="J12" s="131"/>
-      <c r="K12" s="120"/>
+      <c r="I12" s="120"/>
+      <c r="J12" s="132"/>
+      <c r="K12" s="131"/>
       <c r="L12" s="120"/>
       <c r="M12" s="120"/>
       <c r="N12" s="120"/>
@@ -4525,18 +4562,19 @@
       <c r="P12" s="120"/>
       <c r="Q12" s="120"/>
       <c r="R12" s="120"/>
-      <c r="S12" s="132"/>
-      <c r="T12" s="131"/>
-      <c r="U12" s="132"/>
-      <c r="V12" s="131"/>
-      <c r="W12" s="120"/>
+      <c r="S12" s="120"/>
+      <c r="T12" s="132"/>
+      <c r="U12" s="131"/>
+      <c r="V12" s="132"/>
+      <c r="W12" s="131"/>
       <c r="X12" s="120"/>
       <c r="Y12" s="120"/>
       <c r="Z12" s="120"/>
       <c r="AA12" s="120"/>
-      <c r="AB12" s="132"/>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB12" s="120"/>
+      <c r="AC12" s="132"/>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="124" t="s">
         <v>62</v>
       </c>
@@ -4557,54 +4595,55 @@
       <c r="H13" s="120" t="s">
         <v>612</v>
       </c>
-      <c r="I13" s="132" t="s">
+      <c r="I13" s="120" t="s">
         <v>611</v>
       </c>
-      <c r="J13" s="131" t="s">
+      <c r="J13" s="132"/>
+      <c r="K13" s="131" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="120" t="s">
+      <c r="L13" s="120" t="s">
         <v>41</v>
       </c>
-      <c r="L13" s="120" t="s">
+      <c r="M13" s="120" t="s">
         <v>612</v>
       </c>
-      <c r="M13" s="120" t="s">
+      <c r="N13" s="120" t="s">
         <v>22</v>
       </c>
-      <c r="N13" s="120" t="s">
+      <c r="O13" s="120" t="s">
         <v>571</v>
       </c>
-      <c r="O13" s="120" t="s">
+      <c r="P13" s="120" t="s">
         <v>612</v>
       </c>
-      <c r="P13" s="120" t="s">
+      <c r="Q13" s="120" t="s">
         <v>69</v>
-      </c>
-      <c r="Q13" s="120" t="s">
-        <v>22</v>
       </c>
       <c r="R13" s="120" t="s">
         <v>22</v>
       </c>
-      <c r="S13" s="132" t="s">
+      <c r="S13" s="120" t="s">
         <v>22</v>
       </c>
-      <c r="T13" s="131" t="s">
+      <c r="T13" s="132" t="s">
+        <v>22</v>
+      </c>
+      <c r="U13" s="131" t="s">
         <v>576</v>
       </c>
-      <c r="U13" s="132" t="s">
+      <c r="V13" s="132" t="s">
         <v>571</v>
       </c>
-      <c r="V13" s="131"/>
-      <c r="W13" s="120"/>
+      <c r="W13" s="131"/>
       <c r="X13" s="120"/>
       <c r="Y13" s="120"/>
       <c r="Z13" s="120"/>
       <c r="AA13" s="120"/>
-      <c r="AB13" s="132"/>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB13" s="120"/>
+      <c r="AC13" s="132"/>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="124" t="s">
         <v>551</v>
       </c>
@@ -4625,29 +4664,27 @@
       <c r="H14" s="120" t="s">
         <v>553</v>
       </c>
-      <c r="I14" s="132" t="s">
+      <c r="I14" s="120" t="s">
         <v>553</v>
       </c>
-      <c r="J14" s="131" t="s">
+      <c r="J14" s="132"/>
+      <c r="K14" s="131" t="s">
         <v>553</v>
       </c>
-      <c r="K14" s="120" t="s">
+      <c r="L14" s="120" t="s">
         <v>567</v>
       </c>
-      <c r="L14" s="120" t="s">
+      <c r="M14" s="120" t="s">
         <v>569</v>
       </c>
-      <c r="M14" s="120" t="s">
+      <c r="N14" s="120" t="s">
         <v>553</v>
       </c>
-      <c r="N14" s="120" t="s">
+      <c r="O14" s="120" t="s">
         <v>569</v>
       </c>
-      <c r="O14" s="120" t="s">
+      <c r="P14" s="120" t="s">
         <v>567</v>
-      </c>
-      <c r="P14" s="120" t="s">
-        <v>553</v>
       </c>
       <c r="Q14" s="120" t="s">
         <v>553</v>
@@ -4655,24 +4692,27 @@
       <c r="R14" s="120" t="s">
         <v>553</v>
       </c>
-      <c r="S14" s="132" t="s">
+      <c r="S14" s="120" t="s">
         <v>553</v>
       </c>
-      <c r="T14" s="131" t="s">
+      <c r="T14" s="132" t="s">
+        <v>553</v>
+      </c>
+      <c r="U14" s="131" t="s">
         <v>567</v>
       </c>
-      <c r="U14" s="132" t="s">
+      <c r="V14" s="132" t="s">
         <v>569</v>
       </c>
-      <c r="V14" s="131"/>
-      <c r="W14" s="120"/>
+      <c r="W14" s="131"/>
       <c r="X14" s="120"/>
       <c r="Y14" s="120"/>
       <c r="Z14" s="120"/>
       <c r="AA14" s="120"/>
-      <c r="AB14" s="132"/>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB14" s="120"/>
+      <c r="AC14" s="132"/>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="124" t="s">
         <v>552</v>
       </c>
@@ -4693,29 +4733,27 @@
       <c r="H15" s="120" t="s">
         <v>554</v>
       </c>
-      <c r="I15" s="132" t="s">
+      <c r="I15" s="120" t="s">
         <v>554</v>
       </c>
-      <c r="J15" s="131" t="s">
+      <c r="J15" s="132"/>
+      <c r="K15" s="131" t="s">
         <v>554</v>
       </c>
-      <c r="K15" s="120" t="s">
+      <c r="L15" s="120" t="s">
         <v>568</v>
       </c>
-      <c r="L15" s="120" t="s">
+      <c r="M15" s="120" t="s">
         <v>570</v>
       </c>
-      <c r="M15" s="120" t="s">
+      <c r="N15" s="120" t="s">
         <v>554</v>
       </c>
-      <c r="N15" s="120" t="s">
+      <c r="O15" s="120" t="s">
         <v>570</v>
       </c>
-      <c r="O15" s="120" t="s">
+      <c r="P15" s="120" t="s">
         <v>568</v>
-      </c>
-      <c r="P15" s="120" t="s">
-        <v>554</v>
       </c>
       <c r="Q15" s="120" t="s">
         <v>554</v>
@@ -4723,24 +4761,27 @@
       <c r="R15" s="120" t="s">
         <v>554</v>
       </c>
-      <c r="S15" s="132" t="s">
+      <c r="S15" s="120" t="s">
         <v>554</v>
       </c>
-      <c r="T15" s="131" t="s">
+      <c r="T15" s="132" t="s">
+        <v>554</v>
+      </c>
+      <c r="U15" s="131" t="s">
         <v>568</v>
       </c>
-      <c r="U15" s="132" t="s">
+      <c r="V15" s="132" t="s">
         <v>570</v>
       </c>
-      <c r="V15" s="131"/>
-      <c r="W15" s="120"/>
+      <c r="W15" s="131"/>
       <c r="X15" s="120"/>
       <c r="Y15" s="120"/>
       <c r="Z15" s="120"/>
       <c r="AA15" s="120"/>
-      <c r="AB15" s="132"/>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB15" s="120"/>
+      <c r="AC15" s="132"/>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="124" t="s">
         <v>64</v>
       </c>
@@ -4761,54 +4802,55 @@
       <c r="H16" s="120" t="s">
         <v>283</v>
       </c>
-      <c r="I16" s="132" t="s">
+      <c r="I16" s="120" t="s">
         <v>687</v>
       </c>
-      <c r="J16" s="131" t="s">
+      <c r="J16" s="132"/>
+      <c r="K16" s="131" t="s">
         <v>71</v>
       </c>
-      <c r="K16" s="120" t="s">
+      <c r="L16" s="120" t="s">
         <v>72</v>
       </c>
-      <c r="L16" s="120" t="s">
+      <c r="M16" s="120" t="s">
         <v>73</v>
-      </c>
-      <c r="M16" s="120" t="s">
-        <v>278</v>
       </c>
       <c r="N16" s="120" t="s">
         <v>278</v>
       </c>
       <c r="O16" s="120" t="s">
+        <v>278</v>
+      </c>
+      <c r="P16" s="120" t="s">
         <v>71</v>
-      </c>
-      <c r="P16" s="120" t="s">
-        <v>278</v>
       </c>
       <c r="Q16" s="120" t="s">
         <v>278</v>
       </c>
       <c r="R16" s="120" t="s">
+        <v>278</v>
+      </c>
+      <c r="S16" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="S16" s="132" t="s">
+      <c r="T16" s="132" t="s">
         <v>71</v>
       </c>
-      <c r="T16" s="131" t="s">
+      <c r="U16" s="131" t="s">
         <v>687</v>
       </c>
-      <c r="U16" s="132" t="s">
+      <c r="V16" s="132" t="s">
         <v>283</v>
       </c>
-      <c r="V16" s="131"/>
-      <c r="W16" s="120"/>
+      <c r="W16" s="131"/>
       <c r="X16" s="120"/>
       <c r="Y16" s="120"/>
       <c r="Z16" s="120"/>
       <c r="AA16" s="120"/>
-      <c r="AB16" s="132"/>
-    </row>
-    <row r="17" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+      <c r="AB16" s="120"/>
+      <c r="AC16" s="132"/>
+    </row>
+    <row r="17" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="133" t="s">
         <v>593</v>
       </c>
@@ -4819,9 +4861,9 @@
       <c r="F17" s="127"/>
       <c r="G17" s="122"/>
       <c r="H17" s="122"/>
-      <c r="I17" s="128"/>
-      <c r="J17" s="127"/>
-      <c r="K17" s="122"/>
+      <c r="I17" s="122"/>
+      <c r="J17" s="128"/>
+      <c r="K17" s="127"/>
       <c r="L17" s="122"/>
       <c r="M17" s="122"/>
       <c r="N17" s="122"/>
@@ -4829,18 +4871,19 @@
       <c r="P17" s="122"/>
       <c r="Q17" s="122"/>
       <c r="R17" s="122"/>
-      <c r="S17" s="128"/>
-      <c r="T17" s="127"/>
-      <c r="U17" s="128"/>
-      <c r="V17" s="127"/>
-      <c r="W17" s="122"/>
+      <c r="S17" s="122"/>
+      <c r="T17" s="128"/>
+      <c r="U17" s="127"/>
+      <c r="V17" s="128"/>
+      <c r="W17" s="127"/>
       <c r="X17" s="122"/>
       <c r="Y17" s="122"/>
       <c r="Z17" s="122"/>
       <c r="AA17" s="122"/>
-      <c r="AB17" s="128"/>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB17" s="122"/>
+      <c r="AC17" s="128"/>
+    </row>
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="124" t="s">
         <v>584</v>
       </c>
@@ -4851,9 +4894,9 @@
       <c r="F18" s="131"/>
       <c r="G18" s="120"/>
       <c r="H18" s="120"/>
-      <c r="I18" s="132"/>
-      <c r="J18" s="131"/>
-      <c r="K18" s="120"/>
+      <c r="I18" s="120"/>
+      <c r="J18" s="132"/>
+      <c r="K18" s="131"/>
       <c r="L18" s="120"/>
       <c r="M18" s="120"/>
       <c r="N18" s="120"/>
@@ -4861,18 +4904,19 @@
       <c r="P18" s="120"/>
       <c r="Q18" s="120"/>
       <c r="R18" s="120"/>
-      <c r="S18" s="132"/>
-      <c r="T18" s="131"/>
-      <c r="U18" s="132"/>
-      <c r="V18" s="131"/>
-      <c r="W18" s="120"/>
+      <c r="S18" s="120"/>
+      <c r="T18" s="132"/>
+      <c r="U18" s="131"/>
+      <c r="V18" s="132"/>
+      <c r="W18" s="131"/>
       <c r="X18" s="120"/>
       <c r="Y18" s="120"/>
       <c r="Z18" s="120"/>
       <c r="AA18" s="120"/>
-      <c r="AB18" s="132"/>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB18" s="120"/>
+      <c r="AC18" s="132"/>
+    </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="124" t="s">
         <v>8</v>
       </c>
@@ -4883,9 +4927,9 @@
       <c r="F19" s="131"/>
       <c r="G19" s="120"/>
       <c r="H19" s="120"/>
-      <c r="I19" s="132"/>
-      <c r="J19" s="131"/>
-      <c r="K19" s="120"/>
+      <c r="I19" s="120"/>
+      <c r="J19" s="132"/>
+      <c r="K19" s="131"/>
       <c r="L19" s="120"/>
       <c r="M19" s="120"/>
       <c r="N19" s="120"/>
@@ -4893,22 +4937,23 @@
       <c r="P19" s="120"/>
       <c r="Q19" s="120"/>
       <c r="R19" s="120"/>
-      <c r="S19" s="132"/>
-      <c r="T19" s="131">
+      <c r="S19" s="120"/>
+      <c r="T19" s="132"/>
+      <c r="U19" s="131">
         <v>0.5</v>
       </c>
-      <c r="U19" s="132">
+      <c r="V19" s="132">
         <v>0.6</v>
       </c>
-      <c r="V19" s="131"/>
-      <c r="W19" s="120"/>
+      <c r="W19" s="131"/>
       <c r="X19" s="120"/>
       <c r="Y19" s="120"/>
       <c r="Z19" s="120"/>
       <c r="AA19" s="120"/>
-      <c r="AB19" s="132"/>
-    </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB19" s="120"/>
+      <c r="AC19" s="132"/>
+    </row>
+    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="124" t="s">
         <v>560</v>
       </c>
@@ -4919,9 +4964,9 @@
       <c r="F20" s="131"/>
       <c r="G20" s="120"/>
       <c r="H20" s="120"/>
-      <c r="I20" s="132"/>
-      <c r="J20" s="131"/>
-      <c r="K20" s="120"/>
+      <c r="I20" s="120"/>
+      <c r="J20" s="132"/>
+      <c r="K20" s="131"/>
       <c r="L20" s="120"/>
       <c r="M20" s="120"/>
       <c r="N20" s="120"/>
@@ -4929,18 +4974,19 @@
       <c r="P20" s="120"/>
       <c r="Q20" s="120"/>
       <c r="R20" s="120"/>
-      <c r="S20" s="132"/>
-      <c r="T20" s="131"/>
-      <c r="U20" s="132"/>
-      <c r="V20" s="131"/>
-      <c r="W20" s="120"/>
+      <c r="S20" s="120"/>
+      <c r="T20" s="132"/>
+      <c r="U20" s="131"/>
+      <c r="V20" s="132"/>
+      <c r="W20" s="131"/>
       <c r="X20" s="120"/>
       <c r="Y20" s="120"/>
       <c r="Z20" s="120"/>
       <c r="AA20" s="120"/>
-      <c r="AB20" s="132"/>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB20" s="120"/>
+      <c r="AC20" s="132"/>
+    </row>
+    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="116" t="s">
         <v>592</v>
       </c>
@@ -4951,9 +4997,9 @@
       <c r="F21" s="127"/>
       <c r="G21" s="122"/>
       <c r="H21" s="122"/>
-      <c r="I21" s="128"/>
-      <c r="J21" s="127"/>
-      <c r="K21" s="122"/>
+      <c r="I21" s="122"/>
+      <c r="J21" s="128"/>
+      <c r="K21" s="127"/>
       <c r="L21" s="122"/>
       <c r="M21" s="122"/>
       <c r="N21" s="122"/>
@@ -4961,18 +5007,19 @@
       <c r="P21" s="122"/>
       <c r="Q21" s="122"/>
       <c r="R21" s="122"/>
-      <c r="S21" s="128"/>
-      <c r="T21" s="127"/>
-      <c r="U21" s="128"/>
-      <c r="V21" s="127"/>
-      <c r="W21" s="122"/>
+      <c r="S21" s="122"/>
+      <c r="T21" s="128"/>
+      <c r="U21" s="127"/>
+      <c r="V21" s="128"/>
+      <c r="W21" s="127"/>
       <c r="X21" s="122"/>
       <c r="Y21" s="122"/>
       <c r="Z21" s="122"/>
       <c r="AA21" s="122"/>
-      <c r="AB21" s="128"/>
-    </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB21" s="122"/>
+      <c r="AC21" s="128"/>
+    </row>
+    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="124" t="s">
         <v>557</v>
       </c>
@@ -4983,9 +5030,9 @@
       <c r="F22" s="131"/>
       <c r="G22" s="120"/>
       <c r="H22" s="120"/>
-      <c r="I22" s="132"/>
-      <c r="J22" s="131"/>
-      <c r="K22" s="120"/>
+      <c r="I22" s="120"/>
+      <c r="J22" s="132"/>
+      <c r="K22" s="131"/>
       <c r="L22" s="120"/>
       <c r="M22" s="120"/>
       <c r="N22" s="120"/>
@@ -4993,18 +5040,19 @@
       <c r="P22" s="120"/>
       <c r="Q22" s="120"/>
       <c r="R22" s="120"/>
-      <c r="S22" s="132"/>
-      <c r="T22" s="131"/>
-      <c r="U22" s="132"/>
-      <c r="V22" s="131"/>
-      <c r="W22" s="120"/>
+      <c r="S22" s="120"/>
+      <c r="T22" s="132"/>
+      <c r="U22" s="131"/>
+      <c r="V22" s="132"/>
+      <c r="W22" s="131"/>
       <c r="X22" s="120"/>
       <c r="Y22" s="120"/>
       <c r="Z22" s="120"/>
       <c r="AA22" s="120"/>
-      <c r="AB22" s="132"/>
-    </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB22" s="120"/>
+      <c r="AC22" s="132"/>
+    </row>
+    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="124" t="s">
         <v>558</v>
       </c>
@@ -5015,9 +5063,9 @@
       <c r="F23" s="131"/>
       <c r="G23" s="120"/>
       <c r="H23" s="120"/>
-      <c r="I23" s="132"/>
-      <c r="J23" s="131"/>
-      <c r="K23" s="120"/>
+      <c r="I23" s="120"/>
+      <c r="J23" s="132"/>
+      <c r="K23" s="131"/>
       <c r="L23" s="120"/>
       <c r="M23" s="120"/>
       <c r="N23" s="120"/>
@@ -5025,18 +5073,19 @@
       <c r="P23" s="120"/>
       <c r="Q23" s="120"/>
       <c r="R23" s="120"/>
-      <c r="S23" s="132"/>
-      <c r="T23" s="131"/>
-      <c r="U23" s="132"/>
-      <c r="V23" s="131"/>
-      <c r="W23" s="120"/>
+      <c r="S23" s="120"/>
+      <c r="T23" s="132"/>
+      <c r="U23" s="131"/>
+      <c r="V23" s="132"/>
+      <c r="W23" s="131"/>
       <c r="X23" s="120"/>
       <c r="Y23" s="120"/>
       <c r="Z23" s="120"/>
       <c r="AA23" s="120"/>
-      <c r="AB23" s="132"/>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB23" s="120"/>
+      <c r="AC23" s="132"/>
+    </row>
+    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="124" t="s">
         <v>556</v>
       </c>
@@ -5047,9 +5096,9 @@
       <c r="F24" s="131"/>
       <c r="G24" s="120"/>
       <c r="H24" s="120"/>
-      <c r="I24" s="132"/>
-      <c r="J24" s="131"/>
-      <c r="K24" s="120"/>
+      <c r="I24" s="120"/>
+      <c r="J24" s="132"/>
+      <c r="K24" s="131"/>
       <c r="L24" s="120"/>
       <c r="M24" s="120"/>
       <c r="N24" s="120"/>
@@ -5057,18 +5106,19 @@
       <c r="P24" s="120"/>
       <c r="Q24" s="120"/>
       <c r="R24" s="120"/>
-      <c r="S24" s="132"/>
-      <c r="T24" s="131"/>
-      <c r="U24" s="132"/>
-      <c r="V24" s="131"/>
-      <c r="W24" s="120"/>
+      <c r="S24" s="120"/>
+      <c r="T24" s="132"/>
+      <c r="U24" s="131"/>
+      <c r="V24" s="132"/>
+      <c r="W24" s="131"/>
       <c r="X24" s="120"/>
       <c r="Y24" s="120"/>
       <c r="Z24" s="120"/>
       <c r="AA24" s="120"/>
-      <c r="AB24" s="132"/>
-    </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB24" s="120"/>
+      <c r="AC24" s="132"/>
+    </row>
+    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="124" t="s">
         <v>561</v>
       </c>
@@ -5079,9 +5129,9 @@
       <c r="F25" s="131"/>
       <c r="G25" s="120"/>
       <c r="H25" s="120"/>
-      <c r="I25" s="132"/>
-      <c r="J25" s="131"/>
-      <c r="K25" s="120"/>
+      <c r="I25" s="120"/>
+      <c r="J25" s="132"/>
+      <c r="K25" s="131"/>
       <c r="L25" s="120"/>
       <c r="M25" s="120"/>
       <c r="N25" s="120"/>
@@ -5089,18 +5139,19 @@
       <c r="P25" s="120"/>
       <c r="Q25" s="120"/>
       <c r="R25" s="120"/>
-      <c r="S25" s="132"/>
-      <c r="T25" s="131"/>
-      <c r="U25" s="132"/>
-      <c r="V25" s="131"/>
-      <c r="W25" s="120"/>
+      <c r="S25" s="120"/>
+      <c r="T25" s="132"/>
+      <c r="U25" s="131"/>
+      <c r="V25" s="132"/>
+      <c r="W25" s="131"/>
       <c r="X25" s="120"/>
       <c r="Y25" s="120"/>
       <c r="Z25" s="120"/>
       <c r="AA25" s="120"/>
-      <c r="AB25" s="132"/>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB25" s="120"/>
+      <c r="AC25" s="132"/>
+    </row>
+    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="124" t="s">
         <v>559</v>
       </c>
@@ -5111,9 +5162,9 @@
       <c r="F26" s="131"/>
       <c r="G26" s="120"/>
       <c r="H26" s="120"/>
-      <c r="I26" s="132"/>
-      <c r="J26" s="131"/>
-      <c r="K26" s="120"/>
+      <c r="I26" s="120"/>
+      <c r="J26" s="132"/>
+      <c r="K26" s="131"/>
       <c r="L26" s="120"/>
       <c r="M26" s="120"/>
       <c r="N26" s="120"/>
@@ -5121,24 +5172,25 @@
       <c r="P26" s="120"/>
       <c r="Q26" s="120"/>
       <c r="R26" s="120"/>
-      <c r="S26" s="132"/>
-      <c r="T26" s="131"/>
-      <c r="U26" s="132"/>
-      <c r="V26" s="131"/>
-      <c r="W26" s="120"/>
+      <c r="S26" s="120"/>
+      <c r="T26" s="132"/>
+      <c r="U26" s="131"/>
+      <c r="V26" s="132"/>
+      <c r="W26" s="131"/>
       <c r="X26" s="120"/>
       <c r="Y26" s="120"/>
       <c r="Z26" s="120"/>
       <c r="AA26" s="120"/>
-      <c r="AB26" s="132"/>
+      <c r="AB26" s="120"/>
+      <c r="AC26" s="132"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="V1:AB1"/>
-    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="W1:AC1"/>
+    <mergeCell ref="F1:J1"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="J1:S1"/>
-    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="K1:T1"/>
+    <mergeCell ref="U1:V1"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -28979,7 +29031,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:F238"/>
+  <dimension ref="A1:F232"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" style="12" customWidth="1"/>
@@ -32444,176 +32496,88 @@
         <v>144</v>
       </c>
       <c r="B227" s="33">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C227" s="30" t="s">
-        <v>149</v>
+        <v>802</v>
       </c>
       <c r="D227" s="30" t="s">
-        <v>696</v>
-      </c>
-      <c r="E227" s="30"/>
-      <c r="F227" s="30"/>
+        <v>692</v>
+      </c>
+      <c r="E227" s="30" t="s">
+        <v>801</v>
+      </c>
+      <c r="F227" s="30" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="228" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A228" s="31" t="s">
         <v>144</v>
       </c>
       <c r="B228" s="33">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C228" s="31" t="s">
-        <v>150</v>
+        <v>802</v>
       </c>
       <c r="D228" s="30" t="s">
-        <v>696</v>
-      </c>
-      <c r="E228" s="31"/>
-      <c r="F228" s="31"/>
+        <v>692</v>
+      </c>
+      <c r="E228" s="31" t="s">
+        <v>801</v>
+      </c>
+      <c r="F228" s="31" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="229" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A229" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="B229" s="33">
-        <v>4</v>
-      </c>
-      <c r="C229" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="D229" s="30" t="s">
-        <v>696</v>
-      </c>
-      <c r="E229" s="31"/>
-      <c r="F229" s="31"/>
+      <c r="A229" s="24" t="s">
+        <v>155</v>
+      </c>
+      <c r="B229" s="24" t="s">
+        <v>804</v>
+      </c>
+      <c r="C229" s="25"/>
+      <c r="D229" s="25"/>
+      <c r="E229" s="25"/>
+      <c r="F229" s="25"/>
     </row>
     <row r="230" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A230" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="B230" s="33">
-        <v>4</v>
-      </c>
-      <c r="C230" s="31" t="s">
-        <v>152</v>
-      </c>
-      <c r="D230" s="30" t="s">
-        <v>696</v>
-      </c>
-      <c r="E230" s="31"/>
-      <c r="F230" s="31"/>
-    </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A231" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="B231" s="33">
-        <v>0.25</v>
-      </c>
-      <c r="C231" s="31" t="s">
-        <v>153</v>
-      </c>
-      <c r="D231" s="30" t="s">
-        <v>696</v>
-      </c>
-      <c r="E231" s="31"/>
-      <c r="F231" s="31"/>
-    </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A232" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="B232" s="33">
-        <v>0.25</v>
-      </c>
-      <c r="C232" s="31" t="s">
-        <v>154</v>
-      </c>
-      <c r="D232" s="30" t="s">
-        <v>696</v>
-      </c>
-      <c r="E232" s="31"/>
-      <c r="F232" s="31"/>
-    </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A233" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="B233" s="33">
-        <v>0.25</v>
-      </c>
-      <c r="C233" s="31" t="s">
-        <v>266</v>
-      </c>
-      <c r="D233" s="30" t="s">
-        <v>696</v>
-      </c>
-      <c r="E233" s="31"/>
-      <c r="F233" s="31"/>
-    </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A234" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="B234" s="33">
-        <v>0.25</v>
-      </c>
-      <c r="C234" s="31" t="s">
-        <v>267</v>
-      </c>
-      <c r="D234" s="30" t="s">
-        <v>696</v>
-      </c>
-      <c r="E234" s="31"/>
-      <c r="F234" s="31"/>
-    </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A235" s="24" t="s">
-        <v>155</v>
-      </c>
-      <c r="B235" s="24" t="s">
-        <v>159</v>
-      </c>
-      <c r="C235" s="25"/>
-      <c r="D235" s="25"/>
-      <c r="E235" s="25"/>
-      <c r="F235" s="25"/>
-    </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A236" s="24" t="s">
+      <c r="A230" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="B236" s="24" t="s">
-        <v>158</v>
-      </c>
-      <c r="C236" s="25"/>
-      <c r="D236" s="25"/>
-      <c r="E236" s="25"/>
-      <c r="F236" s="25"/>
-    </row>
-    <row r="237" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A237" s="28" t="s">
+      <c r="B230" s="24" t="s">
+        <v>804</v>
+      </c>
+      <c r="C230" s="25"/>
+      <c r="D230" s="25"/>
+      <c r="E230" s="25"/>
+      <c r="F230" s="25"/>
+    </row>
+    <row r="231" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A231" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="B237" s="28" t="s">
-        <v>588</v>
-      </c>
-      <c r="C237" s="29"/>
-      <c r="D237" s="29"/>
-      <c r="E237" s="29"/>
-      <c r="F237" s="29"/>
-    </row>
-    <row r="238" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A238" s="32" t="s">
+      <c r="B231" s="28" t="s">
+        <v>803</v>
+      </c>
+      <c r="C231" s="29"/>
+      <c r="D231" s="29"/>
+      <c r="E231" s="29"/>
+      <c r="F231" s="29"/>
+    </row>
+    <row r="232" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A232" s="32" t="s">
         <v>161</v>
       </c>
-      <c r="B238" s="32" t="s">
+      <c r="B232" s="32" t="s">
         <v>160</v>
       </c>
-      <c r="C238" s="29"/>
-      <c r="D238" s="29"/>
-      <c r="E238" s="29"/>
-      <c r="F238" s="29"/>
+      <c r="C232" s="29"/>
+      <c r="D232" s="29"/>
+      <c r="E232" s="29"/>
+      <c r="F232" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update validation spreadsheets to use a comparison formula rather than an enum/value
Remaining work:
Complete configuration support
Check/Test formula's with multiple expressions (and/or)
Check/Test ranges
Support Towards x From y comparison formula
</commit_message>
<xml_diff>
--- a/data/Data.xlsx
+++ b/data/Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{687CD05D-E31A-4B86-B6F4-991420C95501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2FBF169-17B4-4200-A2A7-5B42FDA753AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26460" yWindow="2205" windowWidth="26100" windowHeight="24405" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patients" sheetId="6" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="Configuration" sheetId="12" r:id="rId8"/>
     <sheet name="Tissue" sheetId="13" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5491" uniqueCount="805">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5455" uniqueCount="787">
   <si>
     <t>Name</t>
   </si>
@@ -2392,61 +2392,7 @@
     <t>2000 s</t>
   </si>
   <si>
-    <t>CSTARS</t>
-  </si>
-  <si>
-    <t>CSTARS-Patient1</t>
-  </si>
-  <si>
-    <t>CSTARS-Patient2</t>
-  </si>
-  <si>
-    <t>CSTARS-Patient3</t>
-  </si>
-  <si>
-    <t>CSTARS-Patient4</t>
-  </si>
-  <si>
-    <t>CSTARS-Patient5</t>
-  </si>
-  <si>
-    <t>CSTARS-Patient6</t>
-  </si>
-  <si>
-    <t>CSTARS-Patient7</t>
-  </si>
-  <si>
-    <t>196 lb</t>
-  </si>
-  <si>
-    <t>54 yr</t>
-  </si>
-  <si>
-    <t>75 in</t>
-  </si>
-  <si>
-    <t>138 lb</t>
-  </si>
-  <si>
-    <t>65 in</t>
-  </si>
-  <si>
-    <t>69 in</t>
-  </si>
-  <si>
-    <t>67 in</t>
-  </si>
-  <si>
     <t>62 yr</t>
-  </si>
-  <si>
-    <t>202 lb</t>
-  </si>
-  <si>
-    <t>200 lb</t>
-  </si>
-  <si>
-    <t>74 in</t>
   </si>
   <si>
     <t>Ventilated</t>
@@ -3847,7 +3793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC26"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.5703125" style="117" bestFit="1" customWidth="1"/>
@@ -3868,11 +3814,10 @@
     <col min="17" max="20" width="10.7109375" style="121" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="15.140625" style="121" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="12.85546875" style="121" bestFit="1" customWidth="1"/>
-    <col min="23" max="29" width="15.85546875" style="121" bestFit="1" customWidth="1"/>
-    <col min="30" max="16384" width="8.85546875" style="121"/>
+    <col min="23" max="16384" width="8.85546875" style="121"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="116"/>
       <c r="B1" s="156" t="s">
         <v>583</v>
@@ -3903,17 +3848,8 @@
         <v>582</v>
       </c>
       <c r="V1" s="158"/>
-      <c r="W1" s="156" t="s">
-        <v>780</v>
-      </c>
-      <c r="X1" s="157"/>
-      <c r="Y1" s="157"/>
-      <c r="Z1" s="157"/>
-      <c r="AA1" s="157"/>
-      <c r="AB1" s="157"/>
-      <c r="AC1" s="158"/>
-    </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="117" t="s">
         <v>0</v>
       </c>
@@ -3942,7 +3878,7 @@
         <v>610</v>
       </c>
       <c r="J2" s="126" t="s">
-        <v>799</v>
+        <v>781</v>
       </c>
       <c r="K2" s="125" t="s">
         <v>25</v>
@@ -3980,29 +3916,8 @@
       <c r="V2" s="126" t="s">
         <v>575</v>
       </c>
-      <c r="W2" s="125" t="s">
-        <v>781</v>
-      </c>
-      <c r="X2" s="125" t="s">
-        <v>782</v>
-      </c>
-      <c r="Y2" s="125" t="s">
-        <v>783</v>
-      </c>
-      <c r="Z2" s="125" t="s">
-        <v>784</v>
-      </c>
-      <c r="AA2" s="125" t="s">
-        <v>785</v>
-      </c>
-      <c r="AB2" s="125" t="s">
-        <v>786</v>
-      </c>
-      <c r="AC2" s="125" t="s">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="116" t="s">
         <v>562</v>
       </c>
@@ -4027,15 +3942,8 @@
       <c r="T3" s="128"/>
       <c r="U3" s="127"/>
       <c r="V3" s="128"/>
-      <c r="W3" s="127"/>
-      <c r="X3" s="122"/>
-      <c r="Y3" s="122"/>
-      <c r="Z3" s="122"/>
-      <c r="AA3" s="122"/>
-      <c r="AB3" s="122"/>
-      <c r="AC3" s="128"/>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="123" t="s">
         <v>409</v>
       </c>
@@ -4102,29 +4010,8 @@
       <c r="V4" s="130" t="s">
         <v>9</v>
       </c>
-      <c r="W4" s="129" t="s">
-        <v>9</v>
-      </c>
-      <c r="X4" s="129" t="s">
-        <v>9</v>
-      </c>
-      <c r="Y4" s="129" t="s">
-        <v>30</v>
-      </c>
-      <c r="Z4" s="129" t="s">
-        <v>9</v>
-      </c>
-      <c r="AA4" s="129" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB4" s="129" t="s">
-        <v>9</v>
-      </c>
-      <c r="AC4" s="129" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="116" t="s">
         <v>590</v>
       </c>
@@ -4149,15 +4036,8 @@
       <c r="T5" s="128"/>
       <c r="U5" s="127"/>
       <c r="V5" s="128"/>
-      <c r="W5" s="127"/>
-      <c r="X5" s="122"/>
-      <c r="Y5" s="122"/>
-      <c r="Z5" s="122"/>
-      <c r="AA5" s="122"/>
-      <c r="AB5" s="122"/>
-      <c r="AC5" s="128"/>
-    </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="124" t="s">
         <v>5</v>
       </c>
@@ -4182,7 +4062,7 @@
         <v>19</v>
       </c>
       <c r="J6" s="132" t="s">
-        <v>795</v>
+        <v>780</v>
       </c>
       <c r="K6" s="131" t="s">
         <v>31</v>
@@ -4220,29 +4100,8 @@
       <c r="V6" s="132" t="s">
         <v>577</v>
       </c>
-      <c r="W6" s="131" t="s">
-        <v>299</v>
-      </c>
-      <c r="X6" s="120" t="s">
-        <v>795</v>
-      </c>
-      <c r="Y6" s="120" t="s">
-        <v>301</v>
-      </c>
-      <c r="Z6" s="120" t="s">
-        <v>301</v>
-      </c>
-      <c r="AA6" s="120" t="s">
-        <v>34</v>
-      </c>
-      <c r="AB6" s="120" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC6" s="132" t="s">
-        <v>789</v>
-      </c>
-    </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="124" t="s">
         <v>6</v>
       </c>
@@ -4299,29 +4158,8 @@
       </c>
       <c r="U7" s="131"/>
       <c r="V7" s="132"/>
-      <c r="W7" s="131" t="s">
-        <v>797</v>
-      </c>
-      <c r="X7" s="120" t="s">
-        <v>796</v>
-      </c>
-      <c r="Y7" s="120" t="s">
-        <v>21</v>
-      </c>
-      <c r="Z7" s="120" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA7" s="120" t="s">
-        <v>791</v>
-      </c>
-      <c r="AB7" s="120" t="s">
-        <v>573</v>
-      </c>
-      <c r="AC7" s="132" t="s">
-        <v>788</v>
-      </c>
-    </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="124" t="s">
         <v>7</v>
       </c>
@@ -4346,7 +4184,7 @@
         <v>20</v>
       </c>
       <c r="J8" s="132" t="s">
-        <v>800</v>
+        <v>782</v>
       </c>
       <c r="K8" s="131" t="s">
         <v>39</v>
@@ -4384,29 +4222,8 @@
       <c r="V8" s="132" t="s">
         <v>579</v>
       </c>
-      <c r="W8" s="131" t="s">
-        <v>798</v>
-      </c>
-      <c r="X8" s="120" t="s">
-        <v>793</v>
-      </c>
-      <c r="Y8" s="120" t="s">
-        <v>794</v>
-      </c>
-      <c r="Z8" s="120" t="s">
-        <v>793</v>
-      </c>
-      <c r="AA8" s="120" t="s">
-        <v>792</v>
-      </c>
-      <c r="AB8" s="120" t="s">
-        <v>790</v>
-      </c>
-      <c r="AC8" s="132" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="124" t="s">
         <v>162</v>
       </c>
@@ -4467,15 +4284,8 @@
       <c r="V9" s="132">
         <v>0.02</v>
       </c>
-      <c r="W9" s="131"/>
-      <c r="X9" s="120"/>
-      <c r="Y9" s="120"/>
-      <c r="Z9" s="120"/>
-      <c r="AA9" s="120"/>
-      <c r="AB9" s="120"/>
-      <c r="AC9" s="132"/>
-    </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="116" t="s">
         <v>591</v>
       </c>
@@ -4500,15 +4310,8 @@
       <c r="T10" s="128"/>
       <c r="U10" s="127"/>
       <c r="V10" s="128"/>
-      <c r="W10" s="127"/>
-      <c r="X10" s="122"/>
-      <c r="Y10" s="122"/>
-      <c r="Z10" s="122"/>
-      <c r="AA10" s="122"/>
-      <c r="AB10" s="122"/>
-      <c r="AC10" s="128"/>
-    </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="124" t="s">
         <v>589</v>
       </c>
@@ -4533,15 +4336,8 @@
       <c r="T11" s="132"/>
       <c r="U11" s="131"/>
       <c r="V11" s="132"/>
-      <c r="W11" s="131"/>
-      <c r="X11" s="120"/>
-      <c r="Y11" s="120"/>
-      <c r="Z11" s="120"/>
-      <c r="AA11" s="120"/>
-      <c r="AB11" s="120"/>
-      <c r="AC11" s="132"/>
-    </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="124" t="s">
         <v>555</v>
       </c>
@@ -4566,15 +4362,8 @@
       <c r="T12" s="132"/>
       <c r="U12" s="131"/>
       <c r="V12" s="132"/>
-      <c r="W12" s="131"/>
-      <c r="X12" s="120"/>
-      <c r="Y12" s="120"/>
-      <c r="Z12" s="120"/>
-      <c r="AA12" s="120"/>
-      <c r="AB12" s="120"/>
-      <c r="AC12" s="132"/>
-    </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="124" t="s">
         <v>62</v>
       </c>
@@ -4635,15 +4424,8 @@
       <c r="V13" s="132" t="s">
         <v>571</v>
       </c>
-      <c r="W13" s="131"/>
-      <c r="X13" s="120"/>
-      <c r="Y13" s="120"/>
-      <c r="Z13" s="120"/>
-      <c r="AA13" s="120"/>
-      <c r="AB13" s="120"/>
-      <c r="AC13" s="132"/>
-    </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="124" t="s">
         <v>551</v>
       </c>
@@ -4704,15 +4486,8 @@
       <c r="V14" s="132" t="s">
         <v>569</v>
       </c>
-      <c r="W14" s="131"/>
-      <c r="X14" s="120"/>
-      <c r="Y14" s="120"/>
-      <c r="Z14" s="120"/>
-      <c r="AA14" s="120"/>
-      <c r="AB14" s="120"/>
-      <c r="AC14" s="132"/>
-    </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="124" t="s">
         <v>552</v>
       </c>
@@ -4773,15 +4548,8 @@
       <c r="V15" s="132" t="s">
         <v>570</v>
       </c>
-      <c r="W15" s="131"/>
-      <c r="X15" s="120"/>
-      <c r="Y15" s="120"/>
-      <c r="Z15" s="120"/>
-      <c r="AA15" s="120"/>
-      <c r="AB15" s="120"/>
-      <c r="AC15" s="132"/>
-    </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="124" t="s">
         <v>64</v>
       </c>
@@ -4842,15 +4610,8 @@
       <c r="V16" s="132" t="s">
         <v>283</v>
       </c>
-      <c r="W16" s="131"/>
-      <c r="X16" s="120"/>
-      <c r="Y16" s="120"/>
-      <c r="Z16" s="120"/>
-      <c r="AA16" s="120"/>
-      <c r="AB16" s="120"/>
-      <c r="AC16" s="132"/>
-    </row>
-    <row r="17" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="133" t="s">
         <v>593</v>
       </c>
@@ -4875,15 +4636,8 @@
       <c r="T17" s="128"/>
       <c r="U17" s="127"/>
       <c r="V17" s="128"/>
-      <c r="W17" s="127"/>
-      <c r="X17" s="122"/>
-      <c r="Y17" s="122"/>
-      <c r="Z17" s="122"/>
-      <c r="AA17" s="122"/>
-      <c r="AB17" s="122"/>
-      <c r="AC17" s="128"/>
-    </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" s="124" t="s">
         <v>584</v>
       </c>
@@ -4908,15 +4662,8 @@
       <c r="T18" s="132"/>
       <c r="U18" s="131"/>
       <c r="V18" s="132"/>
-      <c r="W18" s="131"/>
-      <c r="X18" s="120"/>
-      <c r="Y18" s="120"/>
-      <c r="Z18" s="120"/>
-      <c r="AA18" s="120"/>
-      <c r="AB18" s="120"/>
-      <c r="AC18" s="132"/>
-    </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" s="124" t="s">
         <v>8</v>
       </c>
@@ -4945,15 +4692,8 @@
       <c r="V19" s="132">
         <v>0.6</v>
       </c>
-      <c r="W19" s="131"/>
-      <c r="X19" s="120"/>
-      <c r="Y19" s="120"/>
-      <c r="Z19" s="120"/>
-      <c r="AA19" s="120"/>
-      <c r="AB19" s="120"/>
-      <c r="AC19" s="132"/>
-    </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" s="124" t="s">
         <v>560</v>
       </c>
@@ -4978,15 +4718,8 @@
       <c r="T20" s="132"/>
       <c r="U20" s="131"/>
       <c r="V20" s="132"/>
-      <c r="W20" s="131"/>
-      <c r="X20" s="120"/>
-      <c r="Y20" s="120"/>
-      <c r="Z20" s="120"/>
-      <c r="AA20" s="120"/>
-      <c r="AB20" s="120"/>
-      <c r="AC20" s="132"/>
-    </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" s="116" t="s">
         <v>592</v>
       </c>
@@ -5011,15 +4744,8 @@
       <c r="T21" s="128"/>
       <c r="U21" s="127"/>
       <c r="V21" s="128"/>
-      <c r="W21" s="127"/>
-      <c r="X21" s="122"/>
-      <c r="Y21" s="122"/>
-      <c r="Z21" s="122"/>
-      <c r="AA21" s="122"/>
-      <c r="AB21" s="122"/>
-      <c r="AC21" s="128"/>
-    </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" s="124" t="s">
         <v>557</v>
       </c>
@@ -5044,15 +4770,8 @@
       <c r="T22" s="132"/>
       <c r="U22" s="131"/>
       <c r="V22" s="132"/>
-      <c r="W22" s="131"/>
-      <c r="X22" s="120"/>
-      <c r="Y22" s="120"/>
-      <c r="Z22" s="120"/>
-      <c r="AA22" s="120"/>
-      <c r="AB22" s="120"/>
-      <c r="AC22" s="132"/>
-    </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" s="124" t="s">
         <v>558</v>
       </c>
@@ -5077,15 +4796,8 @@
       <c r="T23" s="132"/>
       <c r="U23" s="131"/>
       <c r="V23" s="132"/>
-      <c r="W23" s="131"/>
-      <c r="X23" s="120"/>
-      <c r="Y23" s="120"/>
-      <c r="Z23" s="120"/>
-      <c r="AA23" s="120"/>
-      <c r="AB23" s="120"/>
-      <c r="AC23" s="132"/>
-    </row>
-    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" s="124" t="s">
         <v>556</v>
       </c>
@@ -5110,15 +4822,8 @@
       <c r="T24" s="132"/>
       <c r="U24" s="131"/>
       <c r="V24" s="132"/>
-      <c r="W24" s="131"/>
-      <c r="X24" s="120"/>
-      <c r="Y24" s="120"/>
-      <c r="Z24" s="120"/>
-      <c r="AA24" s="120"/>
-      <c r="AB24" s="120"/>
-      <c r="AC24" s="132"/>
-    </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" s="124" t="s">
         <v>561</v>
       </c>
@@ -5143,15 +4848,8 @@
       <c r="T25" s="132"/>
       <c r="U25" s="131"/>
       <c r="V25" s="132"/>
-      <c r="W25" s="131"/>
-      <c r="X25" s="120"/>
-      <c r="Y25" s="120"/>
-      <c r="Z25" s="120"/>
-      <c r="AA25" s="120"/>
-      <c r="AB25" s="120"/>
-      <c r="AC25" s="132"/>
-    </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" s="124" t="s">
         <v>559</v>
       </c>
@@ -5176,17 +4874,9 @@
       <c r="T26" s="132"/>
       <c r="U26" s="131"/>
       <c r="V26" s="132"/>
-      <c r="W26" s="131"/>
-      <c r="X26" s="120"/>
-      <c r="Y26" s="120"/>
-      <c r="Z26" s="120"/>
-      <c r="AA26" s="120"/>
-      <c r="AB26" s="120"/>
-      <c r="AC26" s="132"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="W1:AC1"/>
+  <mergeCells count="4">
     <mergeCell ref="F1:J1"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="K1:T1"/>
@@ -32499,13 +32189,13 @@
         <v>1</v>
       </c>
       <c r="C227" s="30" t="s">
-        <v>802</v>
+        <v>784</v>
       </c>
       <c r="D227" s="30" t="s">
         <v>692</v>
       </c>
       <c r="E227" s="30" t="s">
-        <v>801</v>
+        <v>783</v>
       </c>
       <c r="F227" s="30" t="s">
         <v>13</v>
@@ -32519,13 +32209,13 @@
         <v>1</v>
       </c>
       <c r="C228" s="31" t="s">
-        <v>802</v>
+        <v>784</v>
       </c>
       <c r="D228" s="30" t="s">
         <v>692</v>
       </c>
       <c r="E228" s="31" t="s">
-        <v>801</v>
+        <v>783</v>
       </c>
       <c r="F228" s="31" t="s">
         <v>12</v>
@@ -32536,7 +32226,7 @@
         <v>155</v>
       </c>
       <c r="B229" s="24" t="s">
-        <v>804</v>
+        <v>786</v>
       </c>
       <c r="C229" s="25"/>
       <c r="D229" s="25"/>
@@ -32548,7 +32238,7 @@
         <v>156</v>
       </c>
       <c r="B230" s="24" t="s">
-        <v>804</v>
+        <v>786</v>
       </c>
       <c r="C230" s="25"/>
       <c r="D230" s="25"/>
@@ -32560,7 +32250,7 @@
         <v>157</v>
       </c>
       <c r="B231" s="28" t="s">
-        <v>803</v>
+        <v>785</v>
       </c>
       <c r="C231" s="29"/>
       <c r="D231" s="29"/>

</xml_diff>